<commit_message>
Write the rest of the v3.2 notes
The entry stopped at the Gage R&R workbook and missed the four commits after
it: the regression template, the jargon glosses, the scaffolding columns coming
out of the preview, and the two harnesses that can fail again.
</commit_message>
<xml_diff>
--- a/templates/30-regression.xlsx
+++ b/templates/30-regression.xlsx
@@ -114,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -160,15 +160,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -4387,23 +4412,23 @@
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B40" s="25">
+      <c r="B40" s="31">
         <f>IFERROR(INDEX(LINEST($F$11:$F$34,$B$11:$E$34,TRUE,TRUE),1,5),"")</f>
         <v/>
       </c>
-      <c r="C40" s="25">
+      <c r="C40" s="31">
         <f>IFERROR(INDEX(LINEST($F$11:$F$34,$B$11:$E$34,TRUE,TRUE),2,5),"")</f>
         <v/>
       </c>
-      <c r="D40" s="25">
+      <c r="D40" s="31">
         <f>IFERROR($B40/$C40,"")</f>
         <v/>
       </c>
-      <c r="E40" s="28">
+      <c r="E40" s="32">
         <f>IFERROR(TDIST(ABS($D40),$B$55,2),"")</f>
         <v/>
       </c>
-      <c r="I40" s="31">
+      <c r="I40" s="33">
         <f>IF($B40="","","Predicted handle time for a contact with every driver at zero — before 17:00, under the limit, a brand-new agent, no transfers. Read it as the starting point the four effects are added to, not as a prediction.")</f>
         <v/>
       </c>
@@ -4414,27 +4439,27 @@
           <t>Raised after 17:00 (1 = yes)</t>
         </is>
       </c>
-      <c r="B41" s="25">
+      <c r="B41" s="31">
         <f>IFERROR(INDEX(LINEST($F$11:$F$34,$B$11:$E$34,TRUE,TRUE),1,4),"")</f>
         <v/>
       </c>
-      <c r="C41" s="25">
+      <c r="C41" s="31">
         <f>IFERROR(INDEX(LINEST($F$11:$F$34,$B$11:$E$34,TRUE,TRUE),2,4),"")</f>
         <v/>
       </c>
-      <c r="D41" s="25">
+      <c r="D41" s="31">
         <f>IFERROR($B41/$C41,"")</f>
         <v/>
       </c>
-      <c r="E41" s="28">
+      <c r="E41" s="32">
         <f>IFERROR(TDIST(ABS($D41),$B$55,2),"")</f>
         <v/>
       </c>
-      <c r="F41" s="25">
+      <c r="F41" s="31">
         <f>IFERROR(1/(1-INDEX(LINEST($B$11:$B$34,$J$11:$L$34,TRUE,TRUE),3,1)),"")</f>
         <v/>
       </c>
-      <c r="G41" s="22">
+      <c r="G41" s="34">
         <f>IFERROR($B41*(MAX($B$11:$B$34)-MIN($B$11:$B$34)),"")</f>
         <v/>
       </c>
@@ -4442,7 +4467,7 @@
         <f>IF($E41="","",IF($E41&gt;=0.05,"NOT PROVEN — cannot be separated from zero",IF(ABS($G41)&lt;$B$7,"REAL BUT TOO SMALL — under the "&amp;TEXT($B$7,"0")&amp;" seconds you set","ACT ON IT — real, and big enough to matter")))</f>
         <v/>
       </c>
-      <c r="I41" s="31">
+      <c r="I41" s="33">
         <f>IF($B41="","","Seconds the after-17:00 flag adds once the other three are held still. Compare it with the p-value beside it before you repeat it out loud.")</f>
         <v/>
       </c>
@@ -4453,27 +4478,27 @@
           <t>Over the $50 authority limit (1 = yes)</t>
         </is>
       </c>
-      <c r="B42" s="25">
+      <c r="B42" s="31">
         <f>IFERROR(INDEX(LINEST($F$11:$F$34,$B$11:$E$34,TRUE,TRUE),1,3),"")</f>
         <v/>
       </c>
-      <c r="C42" s="25">
+      <c r="C42" s="31">
         <f>IFERROR(INDEX(LINEST($F$11:$F$34,$B$11:$E$34,TRUE,TRUE),2,3),"")</f>
         <v/>
       </c>
-      <c r="D42" s="25">
+      <c r="D42" s="31">
         <f>IFERROR($B42/$C42,"")</f>
         <v/>
       </c>
-      <c r="E42" s="28">
+      <c r="E42" s="32">
         <f>IFERROR(TDIST(ABS($D42),$B$55,2),"")</f>
         <v/>
       </c>
-      <c r="F42" s="25">
+      <c r="F42" s="31">
         <f>IFERROR(1/(1-INDEX(LINEST($C$11:$C$34,$M$11:$O$34,TRUE,TRUE),3,1)),"")</f>
         <v/>
       </c>
-      <c r="G42" s="22">
+      <c r="G42" s="34">
         <f>IFERROR($B42*(MAX($C$11:$C$34)-MIN($C$11:$C$34)),"")</f>
         <v/>
       </c>
@@ -4481,7 +4506,7 @@
         <f>IF($E42="","",IF($E42&gt;=0.05,"NOT PROVEN — cannot be separated from zero",IF(ABS($G42)&lt;$B$7,"REAL BUT TOO SMALL — under the "&amp;TEXT($B$7,"0")&amp;" seconds you set","ACT ON IT — real, and big enough to matter")))</f>
         <v/>
       </c>
-      <c r="I42" s="31">
+      <c r="I42" s="33">
         <f>IF($B42="","","Seconds the $50 authority limit adds once the other three are held still. This is the queue, not the money.")</f>
         <v/>
       </c>
@@ -4492,27 +4517,27 @@
           <t>Agent tenure in months</t>
         </is>
       </c>
-      <c r="B43" s="25">
+      <c r="B43" s="31">
         <f>IFERROR(INDEX(LINEST($F$11:$F$34,$B$11:$E$34,TRUE,TRUE),1,2),"")</f>
         <v/>
       </c>
-      <c r="C43" s="25">
+      <c r="C43" s="31">
         <f>IFERROR(INDEX(LINEST($F$11:$F$34,$B$11:$E$34,TRUE,TRUE),2,2),"")</f>
         <v/>
       </c>
-      <c r="D43" s="25">
+      <c r="D43" s="31">
         <f>IFERROR($B43/$C43,"")</f>
         <v/>
       </c>
-      <c r="E43" s="28">
+      <c r="E43" s="32">
         <f>IFERROR(TDIST(ABS($D43),$B$55,2),"")</f>
         <v/>
       </c>
-      <c r="F43" s="25">
+      <c r="F43" s="31">
         <f>IFERROR(1/(1-INDEX(LINEST($D$11:$D$34,$P$11:$R$34,TRUE,TRUE),3,1)),"")</f>
         <v/>
       </c>
-      <c r="G43" s="22">
+      <c r="G43" s="34">
         <f>IFERROR($B43*(MAX($D$11:$D$34)-MIN($D$11:$D$34)),"")</f>
         <v/>
       </c>
@@ -4520,7 +4545,7 @@
         <f>IF($E43="","",IF($E43&gt;=0.05,"NOT PROVEN — cannot be separated from zero",IF(ABS($G43)&lt;$B$7,"REAL BUT TOO SMALL — under the "&amp;TEXT($B$7,"0")&amp;" seconds you set","ACT ON IT — real, and big enough to matter")))</f>
         <v/>
       </c>
-      <c r="I43" s="31">
+      <c r="I43" s="33">
         <f>IF($B43="","","Seconds per extra month of tenure — negative means longer-serving agents are quicker. Small per month, so read the range column, not this one.")</f>
         <v/>
       </c>
@@ -4531,27 +4556,27 @@
           <t>Transfers before resolution</t>
         </is>
       </c>
-      <c r="B44" s="25">
+      <c r="B44" s="31">
         <f>IFERROR(INDEX(LINEST($F$11:$F$34,$B$11:$E$34,TRUE,TRUE),1,1),"")</f>
         <v/>
       </c>
-      <c r="C44" s="25">
+      <c r="C44" s="31">
         <f>IFERROR(INDEX(LINEST($F$11:$F$34,$B$11:$E$34,TRUE,TRUE),2,1),"")</f>
         <v/>
       </c>
-      <c r="D44" s="25">
+      <c r="D44" s="31">
         <f>IFERROR($B44/$C44,"")</f>
         <v/>
       </c>
-      <c r="E44" s="28">
+      <c r="E44" s="32">
         <f>IFERROR(TDIST(ABS($D44),$B$55,2),"")</f>
         <v/>
       </c>
-      <c r="F44" s="25">
+      <c r="F44" s="31">
         <f>IFERROR(1/(1-INDEX(LINEST($E$11:$E$34,$S$11:$U$34,TRUE,TRUE),3,1)),"")</f>
         <v/>
       </c>
-      <c r="G44" s="22">
+      <c r="G44" s="34">
         <f>IFERROR($B44*(MAX($E$11:$E$34)-MIN($E$11:$E$34)),"")</f>
         <v/>
       </c>
@@ -4559,7 +4584,7 @@
         <f>IF($E44="","",IF($E44&gt;=0.05,"NOT PROVEN — cannot be separated from zero",IF(ABS($G44)&lt;$B$7,"REAL BUT TOO SMALL — under the "&amp;TEXT($B$7,"0")&amp;" seconds you set","ACT ON IT — real, and big enough to matter")))</f>
         <v/>
       </c>
-      <c r="I44" s="31">
+      <c r="I44" s="33">
         <f>IF($B44="","","Seconds each extra transfer adds once the other three are held still. Compare it with the 50.7 seconds the single-driver tab gave you.")</f>
         <v/>
       </c>
@@ -4977,30 +5002,30 @@
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B10" s="32" t="n">
+      <c r="B10" s="35" t="n">
         <v>-3.05</v>
       </c>
-      <c r="C10" s="32" t="n">
+      <c r="C10" s="35" t="n">
         <v>0.24</v>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="36" t="inlineStr">
         <is>
           <t>&lt;0.0001</t>
         </is>
       </c>
-      <c r="E10" s="33">
+      <c r="E10" s="37">
         <f>IFERROR(EXP($B10),"")</f>
         <v/>
       </c>
-      <c r="F10" s="33">
+      <c r="F10" s="37">
         <f>IFERROR(EXP($B10-1.96*$C10),"")</f>
         <v/>
       </c>
-      <c r="G10" s="33">
+      <c r="G10" s="37">
         <f>IFERROR(EXP($B10+1.96*$C10),"")</f>
         <v/>
       </c>
-      <c r="H10" s="34">
+      <c r="H10" s="38">
         <f>"Baseline odds of a reopen with every driver at zero: "&amp;TEXT($E10,"0.000")&amp;" to 1, which is "&amp;TEXT($E10/(1+$E10),"0.0%")&amp;" probability."</f>
         <v/>
       </c>
@@ -5011,30 +5036,30 @@
           <t>Raised after 17:00 (1 = yes)</t>
         </is>
       </c>
-      <c r="B11" s="35" t="n">
+      <c r="B11" s="39" t="n">
         <v>1.16</v>
       </c>
-      <c r="C11" s="35" t="n">
+      <c r="C11" s="39" t="n">
         <v>0.21</v>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="40" t="inlineStr">
         <is>
           <t>&lt;0.0001</t>
         </is>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="41">
         <f>IFERROR(EXP($B11),"")</f>
         <v/>
       </c>
-      <c r="F11" s="27">
+      <c r="F11" s="41">
         <f>IFERROR(EXP($B11-1.96*$C11),"")</f>
         <v/>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="41">
         <f>IFERROR(EXP($B11+1.96*$C11),"")</f>
         <v/>
       </c>
-      <c r="H11" s="31">
+      <c r="H11" s="33">
         <f>"Raising the adjustment after 17:00 multiplies the odds of a reopen by "&amp;TEXT($E11,"0.00")&amp;". This is the posting-batch effect, and it is the largest single driver in the model."</f>
         <v/>
       </c>
@@ -5045,30 +5070,30 @@
           <t>Over the $50 authority limit (1 = yes)</t>
         </is>
       </c>
-      <c r="B12" s="35" t="n">
+      <c r="B12" s="39" t="n">
         <v>0.83</v>
       </c>
-      <c r="C12" s="35" t="n">
+      <c r="C12" s="39" t="n">
         <v>0.22</v>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="40" t="inlineStr">
         <is>
           <t>0.0002</t>
         </is>
       </c>
-      <c r="E12" s="27">
+      <c r="E12" s="41">
         <f>IFERROR(EXP($B12),"")</f>
         <v/>
       </c>
-      <c r="F12" s="27">
+      <c r="F12" s="41">
         <f>IFERROR(EXP($B12-1.96*$C12),"")</f>
         <v/>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="41">
         <f>IFERROR(EXP($B12+1.96*$C12),"")</f>
         <v/>
       </c>
-      <c r="H12" s="31">
+      <c r="H12" s="33">
         <f>"Clearing the $50 authority limit multiplies the odds of a reopen by "&amp;TEXT($E12,"0.00")&amp;", because the case waits in a queue for approval."</f>
         <v/>
       </c>
@@ -5079,30 +5104,30 @@
           <t>Agent tenure in months</t>
         </is>
       </c>
-      <c r="B13" s="35" t="n">
+      <c r="B13" s="39" t="n">
         <v>-0.038</v>
       </c>
-      <c r="C13" s="35" t="n">
+      <c r="C13" s="39" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="40" t="inlineStr">
         <is>
           <t>&lt;0.0001</t>
         </is>
       </c>
-      <c r="E13" s="27">
+      <c r="E13" s="41">
         <f>IFERROR(EXP($B13),"")</f>
         <v/>
       </c>
-      <c r="F13" s="27">
+      <c r="F13" s="41">
         <f>IFERROR(EXP($B13-1.96*$C13),"")</f>
         <v/>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="41">
         <f>IFERROR(EXP($B13+1.96*$C13),"")</f>
         <v/>
       </c>
-      <c r="H13" s="31">
+      <c r="H13" s="33">
         <f>"Each extra month of tenure multiplies the odds by "&amp;TEXT($E13,"0.000")&amp;" — so a 24-month agent runs at "&amp;TEXT($E13^24,"0.00")&amp;" times the odds of a first-week agent."</f>
         <v/>
       </c>
@@ -5113,30 +5138,30 @@
           <t>Transfers before resolution</t>
         </is>
       </c>
-      <c r="B14" s="35" t="n">
+      <c r="B14" s="39" t="n">
         <v>0.61</v>
       </c>
-      <c r="C14" s="35" t="n">
+      <c r="C14" s="39" t="n">
         <v>0.12</v>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="40" t="inlineStr">
         <is>
           <t>&lt;0.0001</t>
         </is>
       </c>
-      <c r="E14" s="27">
+      <c r="E14" s="41">
         <f>IFERROR(EXP($B14),"")</f>
         <v/>
       </c>
-      <c r="F14" s="27">
+      <c r="F14" s="41">
         <f>IFERROR(EXP($B14-1.96*$C14),"")</f>
         <v/>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="41">
         <f>IFERROR(EXP($B14+1.96*$C14),"")</f>
         <v/>
       </c>
-      <c r="H14" s="31">
+      <c r="H14" s="33">
         <f>"Each extra transfer multiplies the odds of a reopen by "&amp;TEXT($E14,"0.00")&amp;". Multiply by how common transfers are before you rank it against the others."</f>
         <v/>
       </c>
@@ -5232,15 +5257,15 @@
       <c r="F19" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="33">
+      <c r="G19" s="42">
         <f>IF($B19="","",$B$10+$B$11*$B19+$B$12*$C19+$B$13*$D19+$B$14*$E19)</f>
         <v/>
       </c>
-      <c r="H19" s="36">
+      <c r="H19" s="43">
         <f>IFERROR(1/(1+EXP(-$G19)),"")</f>
         <v/>
       </c>
-      <c r="I19" s="37">
+      <c r="I19" s="44">
         <f>IF($H19="","",IF($H19&gt;=$B$45,1,0))</f>
         <v/>
       </c>
@@ -6055,7 +6080,7 @@
           <t>Flag a contact at this probability or above</t>
         </is>
       </c>
-      <c r="B45" s="38" t="n">
+      <c r="B45" s="45" t="n">
         <v>0.2</v>
       </c>
       <c r="C45" s="10" t="inlineStr">
@@ -6070,7 +6095,7 @@
           <t>AUC the tool reported</t>
         </is>
       </c>
-      <c r="B46" s="39" t="n">
+      <c r="B46" s="46" t="n">
         <v>0.74</v>
       </c>
       <c r="C46" s="10" t="inlineStr">

</xml_diff>